<commit_message>
Excel完全ガイド 2-2-2: ⑨ EOMONTH+SEQUENCE と 問題Q6 を追加
- ⑨「5年分の月初(X月1日)を横スピル」= EOMONTH(基準,SEQUENCE(1,60,0))+1
- 標準/full 両xlsxにデモ⑨と問題Q6を追加（スピル先は空にし#SPILL回避）
- HTMLに⑨行・コード例・EOMONTH補足note・DL説明(①〜⑨/Q1〜Q6)を反映

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/excel-mastery-2-2-2.xlsx
+++ b/files/excel-mastery-2-2-2.xlsx
@@ -2,33 +2,80 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-1605" yWindow="-15870" windowWidth="29040" windowHeight="15990" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="2-2-2_スピル関数" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="6">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy/m/d"/>
+  </numFmts>
+  <fonts count="11">
     <font>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <family val="3"/>
       <b val="1"/>
       <color rgb="FF002060"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <family val="3"/>
+      <color rgb="FFFF0000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <family val="3"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <family val="3"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <family val="3"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <family val="3"/>
+      <sz val="6"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
     </font>
     <font>
       <color rgb="FFFF0000"/>
@@ -36,20 +83,13 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -58,7 +98,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3F51"/>
+        <fgColor rgb="FF1F3F51"/>
       </patternFill>
     </fill>
     <fill>
@@ -76,8 +116,13 @@
         <fgColor rgb="FFFFF6D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3F51"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -98,6 +143,31 @@
       <bottom style="thin">
         <color rgb="FFBFBFBF"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -120,40 +190,27 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
       <top style="thin">
         <color rgb="FFBFBFBF"/>
       </top>
       <bottom style="thin">
         <color rgb="FFBFBFBF"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFBFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFBFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFBFBFBF"/>
-      </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -170,13 +227,27 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="10" fillId="5" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -539,28 +610,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:K130"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:M114"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13"/>
   <cols>
-    <col width="2.4" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="3" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="2.36328125" customWidth="1" style="17" min="1" max="1"/>
+    <col width="11" customWidth="1" style="17" min="2" max="3"/>
+    <col width="16" customWidth="1" style="17" min="4" max="4"/>
+    <col width="9" customWidth="1" style="17" min="5" max="5"/>
+    <col width="12" customWidth="1" style="17" min="6" max="6"/>
+    <col width="3" customWidth="1" style="17" min="7" max="7"/>
+    <col width="16" customWidth="1" style="17" min="8" max="10"/>
+    <col width="14" customWidth="1" style="17" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="2">
+    <row r="1"/>
+    <row r="2" ht="16.5" customHeight="1" s="17">
       <c r="B2" s="1" t="inlineStr">
         <is>
           <t>2-2-2. データ加工・クリーニング ― スピル関数系（UNIQUE / FILTER / SORTBY / TOCOL / TOROW / DROP / TEXTSPLIT / SEQUENCE）</t>
         </is>
       </c>
+      <c r="C2" s="1" t="n"/>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
@@ -568,617 +638,713 @@
           <t>各「数式」セル（青）はExcelで開くと自動計算し、下方向・右方向にスピル（spill）します。※動的配列に対応した Microsoft 365 が必要です。</t>
         </is>
       </c>
-    </row>
+      <c r="C3" s="2" t="n"/>
+    </row>
+    <row r="4"/>
+    <row r="5"/>
     <row r="6">
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>【元データ】予約明細（空白セルと『合計』行をわざと含む）</t>
         </is>
       </c>
+      <c r="H6" s="16" t="inlineStr">
+        <is>
+          <t>① UNIQUE + TOCOL ｜ 空白を集計しない</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>予約ID</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>予約経路ID</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>予約経路</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>区分</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>売上</t>
         </is>
       </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>UNIQUE で重複除去。</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>TOCOL(範囲,1) で1列に畳みつつ空白を無視 → UNIQUE で重複除去。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>R001</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>RC001</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>楽天トラベル</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>国内</t>
         </is>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="F8" s="6" t="n">
         <v>160000</v>
       </c>
+      <c r="H8" s="7">
+        <f t="array" ref="H8:H14">_xlfn.UNIQUE(D:D)</f>
+        <v/>
+      </c>
+      <c r="J8" s="7">
+        <f t="array" ref="J8:J13">_xlfn.UNIQUE(_xlfn.TOCOL(D:D,1))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>R002</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>RC002</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>じゃらん</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>国内</t>
         </is>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="F9" s="6" t="n">
         <v>108000</v>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>R003</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>RC005</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Booking.com</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>海外</t>
         </is>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="F10" s="6" t="n">
         <v>72000</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>R004</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="12" t="n"/>
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>国内</t>
         </is>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="F11" s="6" t="n">
         <v>180000</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>R005</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>RC010</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>公式サイト</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>国内</t>
         </is>
       </c>
-      <c r="E12" s="7" t="n">
+      <c r="F12" s="6" t="n">
         <v>95000</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>R006</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>RC002</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>じゃらん</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>国内</t>
         </is>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="F13" s="6" t="n">
         <v>36000</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>R007</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>RC008</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>Expedia</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>海外</t>
         </is>
       </c>
-      <c r="E14" s="7" t="n">
+      <c r="F14" s="6" t="n">
         <v>152000</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>R008</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="C15" s="4" t="n"/>
+      <c r="D15" s="12" t="n"/>
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>海外</t>
         </is>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="F15" s="6" t="n">
         <v>74000</v>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>R009</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>RC001</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>楽天トラベル</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>国内</t>
         </is>
       </c>
-      <c r="E16" s="7" t="n">
+      <c r="F16" s="6" t="n">
         <v>92000</v>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>合計</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="n">
-        <v>969000</v>
+    <row r="17"/>
+    <row r="18">
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>※ C7がヘッダー、C11・C15 が空白</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n"/>
+      <c r="H18" s="16" t="inlineStr">
+        <is>
+          <t>② UNIQUE + TOCOL + FILTER ｜ 空白＋特定セル(合計)を除外＝実データのみ</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>※ C11・C15 が空白、C17 が『合計』。これらを除いて“実データのみ”を取り出すのが下の例です。</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>① UNIQUE + TOCOL ｜ 空白を集計しない</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>TOCOL(範囲,1) で1列に畳みつつ空白を無視 → UNIQUE で重複除去。</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="8">
-        <f>UNIQUE(TOCOL(C8:C17,1))</f>
+          <t>これらを除いて“実データのみ”を取り出すのが右の例です。</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n"/>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>FILTER で『予約経路』を除外 → TOCOL(,1) で空白無視 → UNIQUE。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="H20" s="7">
+        <f t="array" ref="H20:H24">_xlfn.UNIQUE(_xlfn.TOCOL(_xlfn._xlws.FILTER(D:D,D:D&lt;&gt;"予約経路"),1))</f>
         <v/>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>② UNIQUE + TOCOL + FILTER ｜ 空白＋特定セル(合計)を除外＝実データのみ</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>FILTER で『合計』を除外 → TOCOL(,1) で空白無視 → UNIQUE。</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="8">
-        <f>UNIQUE(TOCOL(FILTER(C8:C17,C8:C17&lt;&gt;"合計"),1))</f>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30">
+      <c r="H30" s="16" t="inlineStr">
+        <is>
+          <t>③ UNIQUE + TOCOL + DROP ｜ 空白＋先頭の任意行を除外</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>DROP(範囲,7) で先頭7行を落とす → TOCOL(,1) → UNIQUE。ヘッダや前置き行を飛ばす用途。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="H32" s="7">
+        <f t="array" ref="H32:H36">_xlfn.UNIQUE(_xlfn.TOCOL(_xlfn.DROP(D:D,7),1))</f>
         <v/>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>③ UNIQUE + TOCOL + DROP ｜ 空白＋先頭の任意行を除外</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>DROP(範囲,3) で先頭3行を落とす → TOCOL(,1) → UNIQUE。ヘッダや前置き行を飛ばす用途。</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" s="8">
-        <f>UNIQUE(TOCOL(DROP(C8:C17,3),1))</f>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42">
+      <c r="H42" s="16" t="inlineStr">
+        <is>
+          <t>④ ③ + SORT ｜ さらに任意の順で並べ替え（ここでは降順）</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>SORT(結果, 並べ替えキーの列番号, -1)。キー配列を差し替えれば任意の順に。</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="H44" s="7">
+        <f t="array" ref="H44:H48">_xlfn._xlws.SORT(_xlfn.UNIQUE(_xlfn.TOCOL(_xlfn.DROP(D:D,7),1)),1,-1)</f>
         <v/>
       </c>
     </row>
-    <row r="58">
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>④ ③ + SORTBY ｜ さらに任意の順で並べ替え（ここでは降順）</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="B59" s="2" t="inlineStr">
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54">
+      <c r="H54" s="16" t="inlineStr">
+        <is>
+          <t>⑤ ③ + SORTBY ｜ さらに任意の順で並べ替え（ここでは昇順）</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="H55" s="2" t="inlineStr">
         <is>
           <t>SORTBY(結果, 並べ替えキー, -1)。キー配列を差し替えれば任意の順に。</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="B60" s="8">
-        <f>SORTBY(UNIQUE(TOCOL(DROP(C8:C17,3),1)),UNIQUE(TOCOL(DROP(C8:C17,3),1)),-1)</f>
+    <row r="56">
+      <c r="H56" s="7">
+        <f t="array" ref="H56:H60">_xlfn.SORTBY(
+                _xlfn.UNIQUE(_xlfn.TOCOL(_xlfn.DROP(C:C,7),1)),
+                _xlfn.UNIQUE(_xlfn.TOCOL(_xlfn.DROP(C:C,7),1)),
+                1
+               )</f>
         <v/>
       </c>
+      <c r="I56" s="7">
+        <f t="array" ref="I56:I60">_xlfn.XLOOKUP(_xlfn.ANCHORARRAY(H56),C:C,D:D)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66">
+      <c r="H66" s="16" t="inlineStr">
+        <is>
+          <t>⑥ TOCOL / TOROW ｜ データの縦横を変換</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>TOCOL＝横→縦、TOROW＝縦→横。貼り付け方向を直したい時に。</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="H68" s="8" t="inlineStr">
+        <is>
+          <t>横入力→</t>
+        </is>
+      </c>
+      <c r="I68" s="9" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="J68" s="9" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="K68" s="9" t="inlineStr">
+        <is>
+          <t>水</t>
+        </is>
+      </c>
+      <c r="L68" s="9" t="inlineStr">
+        <is>
+          <t>木</t>
+        </is>
+      </c>
+      <c r="M68" s="9" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>↓ TOCOL で縦1列に</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>→ TOROW で C8:C10 を横1行に</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>⑤ FILTER + SORTBY ｜ ヘッダー行を除いて抽出→売上の降順</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>参照をB8(見出しの下)から始めるとヘッダーは自然に除外。空白行はFILTERで除外し、SORTBYで売上降順。</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="B72" s="8">
-        <f>SORTBY(FILTER(B8:E16,C8:C16&lt;&gt;""),FILTER(E8:E16,C8:C16&lt;&gt;""),-1)</f>
+      <c r="H70" s="7">
+        <f t="array" ref="H70:H74">_xlfn.TOCOL(I68:M68)</f>
         <v/>
       </c>
+      <c r="J70" s="7">
+        <f t="array" ref="J70:L70">_xlfn.TOROW(D8:D10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80">
+      <c r="H80" s="16" t="inlineStr">
+        <is>
+          <t>⑦ TOCOL + TEXTSPLIT ｜ カンマ区切り文字列を縦1列に</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>web/PDFの表を貼れない時、カンマ区切りテキストを縦のリストに展開できる。</t>
+        </is>
+      </c>
     </row>
     <row r="82">
-      <c r="B82" s="3" t="inlineStr">
-        <is>
-          <t>⑥ TOCOL / TOROW ｜ データの縦横を変換</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="B83" s="2" t="inlineStr">
-        <is>
-          <t>TOCOL＝横→縦、TOROW＝縦→横。貼り付け方向を直したい時に。</t>
-        </is>
-      </c>
-    </row>
+      <c r="H82" s="8" t="inlineStr">
+        <is>
+          <t>入力→</t>
+        </is>
+      </c>
+      <c r="I82" s="10" t="inlineStr">
+        <is>
+          <t>りんご,みかん,ぶどう,いちご,かき</t>
+        </is>
+      </c>
+    </row>
+    <row r="83"/>
     <row r="84">
-      <c r="B84" s="9" t="inlineStr">
-        <is>
-          <t>横入力→</t>
-        </is>
-      </c>
-      <c r="C84" s="10" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="D84" s="10" t="inlineStr">
-        <is>
-          <t>火</t>
-        </is>
-      </c>
-      <c r="E84" s="10" t="inlineStr">
-        <is>
-          <t>水</t>
-        </is>
-      </c>
-      <c r="F84" s="10" t="inlineStr">
-        <is>
-          <t>木</t>
-        </is>
-      </c>
-      <c r="G84" s="10" t="inlineStr">
-        <is>
-          <t>金</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="B85" s="2" t="inlineStr">
-        <is>
-          <t>↓ TOCOL で縦1列に</t>
-        </is>
-      </c>
-      <c r="D85" s="2" t="inlineStr">
-        <is>
-          <t>→ TOROW で C8:C10 を横1行に</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="B86" s="8">
-        <f>TOCOL(C84:G84)</f>
+      <c r="H84" s="7">
+        <f t="array" ref="H84:H88">_xlfn.TOCOL(_xlfn.TEXTSPLIT(I82,","))</f>
         <v/>
       </c>
-      <c r="D86" s="8">
-        <f>TOROW(C8:C10)</f>
+    </row>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94">
+      <c r="H94" s="16" t="inlineStr">
+        <is>
+          <t>⑧ SEQUENCE + ROWS ｜ データ件数ぶんの連番を自動生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>ROWS で件数を数え、その数だけ連番を作る。行が増減しても自動追従。</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="H96" s="7">
+        <f t="array" ref="H96:H100">_xlfn.SEQUENCE(ROWS(_xlfn.ANCHORARRAY(H44)))</f>
         <v/>
       </c>
-    </row>
-    <row r="96">
-      <c r="B96" s="3" t="inlineStr">
-        <is>
-          <t>⑦ TOCOL + TEXTSPLIT ｜ カンマ区切り文字列を縦1列に</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="B97" s="2" t="inlineStr">
-        <is>
-          <t>web/PDFの表を貼れない時、カンマ区切りテキストを縦のリストに展開できる。</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="B98" s="9" t="inlineStr">
-        <is>
-          <t>入力→</t>
-        </is>
-      </c>
-      <c r="C98" s="11" t="inlineStr">
-        <is>
-          <t>りんご,みかん,ぶどう,いちご,かき</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="B100" s="8">
-        <f>TOCOL(TEXTSPLIT(C98,","))</f>
+      <c r="I96" s="7">
+        <f t="array" ref="I96:I100">_xlfn.ANCHORARRAY(H44)</f>
         <v/>
       </c>
     </row>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102">
+      <c r="H102" s="18" t="inlineStr">
+        <is>
+          <t>⑨ EOMONTH + SEQUENCE ｜ 5年分の“月初(X月1日)”を横にスピル</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="H103" s="19" t="inlineStr">
+        <is>
+          <t>SEQUENCE(1,60,0) で 0〜59 か月を作り、EOMONTH(基準,n)+1 で各月の1日に。基準日を変えると全体が動く。</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="H104" s="20" t="inlineStr">
+        <is>
+          <t>基準日→</t>
+        </is>
+      </c>
+      <c r="I104" s="21" t="n">
+        <v>46037</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="H105" s="22">
+        <f>EOMONTH(I104,_xlfn.SEQUENCE(1,60,0))+1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="H106" s="19" t="inlineStr">
+        <is>
+          <t>↑ H105から右へ60列（5年＝60か月）ぶんの月初がスピルします。</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="H107" s="16" t="inlineStr">
+        <is>
+          <t>▼ 問題（黄色セルに自分で数式を入れてみよう。解答は右のI列）</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="H108" s="15" t="inlineStr">
+        <is>
+          <t>問題</t>
+        </is>
+      </c>
+      <c r="I108" s="13" t="n"/>
+      <c r="J108" s="13" t="n"/>
+      <c r="K108" s="13" t="n"/>
+      <c r="L108" s="14" t="n"/>
+      <c r="M108" s="11" t="inlineStr">
+        <is>
+          <t>解答欄</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="H109" s="12" t="inlineStr">
+        <is>
+          <t>Q1  C列から空白を除いた重複なしリストを作る</t>
+        </is>
+      </c>
+      <c r="I109" s="13" t="n"/>
+      <c r="J109" s="13" t="n"/>
+      <c r="K109" s="13" t="n"/>
+      <c r="L109" s="14" t="n"/>
+      <c r="M109" s="10" t="n"/>
+    </row>
     <row r="110">
-      <c r="B110" s="3" t="inlineStr">
-        <is>
-          <t>⑧ SEQUENCE + ROWS ｜ データ件数ぶんの連番を自動生成</t>
-        </is>
-      </c>
+      <c r="H110" s="12" t="inlineStr">
+        <is>
+          <t>Q2  Q1に加えて『合計』も除外し、実データのみのリストにする</t>
+        </is>
+      </c>
+      <c r="I110" s="13" t="n"/>
+      <c r="J110" s="13" t="n"/>
+      <c r="K110" s="13" t="n"/>
+      <c r="L110" s="14" t="n"/>
+      <c r="M110" s="10" t="n"/>
     </row>
     <row r="111">
-      <c r="B111" s="2" t="inlineStr">
-        <is>
-          <t>ROWS で件数を数え、その数だけ連番を作る。行が増減しても自動追従。</t>
-        </is>
-      </c>
+      <c r="H111" s="12" t="inlineStr">
+        <is>
+          <t>Q3  空白でない行だけを抽出し、売上の降順に並べ替える（ヘッダー除く）</t>
+        </is>
+      </c>
+      <c r="I111" s="13" t="n"/>
+      <c r="J111" s="13" t="n"/>
+      <c r="K111" s="13" t="n"/>
+      <c r="L111" s="14" t="n"/>
+      <c r="M111" s="10" t="n"/>
     </row>
     <row r="112">
-      <c r="B112" s="2" t="inlineStr">
-        <is>
-          <t>元データ10行ぶんの連番</t>
-        </is>
-      </c>
-      <c r="D112" s="2" t="inlineStr">
-        <is>
-          <t>②の実データ件数ぶんの連番</t>
-        </is>
-      </c>
+      <c r="H112" s="12" t="inlineStr">
+        <is>
+          <t>Q4  文字列『東京,大阪,名古屋』を縦1列に展開する</t>
+        </is>
+      </c>
+      <c r="I112" s="13" t="n"/>
+      <c r="J112" s="13" t="n"/>
+      <c r="K112" s="13" t="n"/>
+      <c r="L112" s="14" t="n"/>
+      <c r="M112" s="10" t="n"/>
     </row>
     <row r="113">
-      <c r="B113" s="8">
-        <f>SEQUENCE(ROWS(C8:C17))</f>
-        <v/>
-      </c>
-      <c r="D113" s="8">
-        <f>SEQUENCE(ROWS(UNIQUE(TOCOL(FILTER(C8:C17,C8:C17&lt;&gt;"合計"),1))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="124">
-      <c r="B124" s="3" t="inlineStr">
-        <is>
-          <t>▼ 問題（黄色セルに自分で数式を入れてみよう。解答は右のI列）</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="B125" s="12" t="inlineStr">
-        <is>
-          <t>問題</t>
-        </is>
-      </c>
-      <c r="C125" s="13" t="n"/>
-      <c r="D125" s="13" t="n"/>
-      <c r="E125" s="13" t="n"/>
-      <c r="F125" s="14" t="n"/>
-      <c r="G125" s="15" t="inlineStr">
-        <is>
-          <t>解答欄</t>
-        </is>
-      </c>
-      <c r="I125" s="12" t="inlineStr">
-        <is>
-          <t>解答例</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="B126" s="6" t="inlineStr">
-        <is>
-          <t>Q1  C列から空白を除いた重複なしリストを作る</t>
-        </is>
-      </c>
-      <c r="C126" s="13" t="n"/>
-      <c r="D126" s="13" t="n"/>
-      <c r="E126" s="13" t="n"/>
-      <c r="F126" s="14" t="n"/>
-      <c r="G126" s="11" t="n"/>
-      <c r="I126" s="6" t="inlineStr">
-        <is>
-          <t>=UNIQUE(TOCOL(C8:C17,1))</t>
-        </is>
-      </c>
-      <c r="J126" s="13" t="n"/>
-      <c r="K126" s="14" t="n"/>
-    </row>
-    <row r="127">
-      <c r="B127" s="6" t="inlineStr">
-        <is>
-          <t>Q2  Q1に加えて『合計』も除外し、実データのみのリストにする</t>
-        </is>
-      </c>
-      <c r="C127" s="13" t="n"/>
-      <c r="D127" s="13" t="n"/>
-      <c r="E127" s="13" t="n"/>
-      <c r="F127" s="14" t="n"/>
-      <c r="G127" s="11" t="n"/>
-      <c r="I127" s="6" t="inlineStr">
-        <is>
-          <t>=UNIQUE(TOCOL(FILTER(C8:C17,C8:C17&lt;&gt;"合計"),1))</t>
-        </is>
-      </c>
-      <c r="J127" s="13" t="n"/>
-      <c r="K127" s="14" t="n"/>
-    </row>
-    <row r="128">
-      <c r="B128" s="6" t="inlineStr">
-        <is>
-          <t>Q3  空白でない行だけを抽出し、売上の降順に並べ替える（ヘッダー除く）</t>
-        </is>
-      </c>
-      <c r="C128" s="13" t="n"/>
-      <c r="D128" s="13" t="n"/>
-      <c r="E128" s="13" t="n"/>
-      <c r="F128" s="14" t="n"/>
-      <c r="G128" s="11" t="n"/>
-      <c r="I128" s="6" t="inlineStr">
-        <is>
-          <t>=SORTBY(FILTER(B8:E16,C8:C16&lt;&gt;""),FILTER(E8:E16,C8:C16&lt;&gt;""),-1)</t>
-        </is>
-      </c>
-      <c r="J128" s="13" t="n"/>
-      <c r="K128" s="14" t="n"/>
-    </row>
-    <row r="129">
-      <c r="B129" s="6" t="inlineStr">
-        <is>
-          <t>Q4  文字列『東京,大阪,名古屋』を縦1列に展開する</t>
-        </is>
-      </c>
-      <c r="C129" s="13" t="n"/>
-      <c r="D129" s="13" t="n"/>
-      <c r="E129" s="13" t="n"/>
-      <c r="F129" s="14" t="n"/>
-      <c r="G129" s="11" t="n"/>
-      <c r="I129" s="6" t="inlineStr">
-        <is>
-          <t>=TOCOL(TEXTSPLIT("東京,大阪,名古屋",","))</t>
-        </is>
-      </c>
-      <c r="J129" s="13" t="n"/>
-      <c r="K129" s="14" t="n"/>
-    </row>
-    <row r="130">
-      <c r="B130" s="6" t="inlineStr">
+      <c r="H113" s="12" t="inlineStr">
         <is>
           <t>Q5  元データの件数ぶん（10行）の連番を作る</t>
         </is>
       </c>
-      <c r="C130" s="13" t="n"/>
-      <c r="D130" s="13" t="n"/>
-      <c r="E130" s="13" t="n"/>
-      <c r="F130" s="14" t="n"/>
-      <c r="G130" s="11" t="n"/>
-      <c r="I130" s="6" t="inlineStr">
-        <is>
-          <t>=SEQUENCE(ROWS(C8:C17))</t>
-        </is>
-      </c>
-      <c r="J130" s="13" t="n"/>
-      <c r="K130" s="14" t="n"/>
+      <c r="I113" s="13" t="n"/>
+      <c r="J113" s="13" t="n"/>
+      <c r="K113" s="13" t="n"/>
+      <c r="L113" s="14" t="n"/>
+      <c r="M113" s="10" t="n"/>
+    </row>
+    <row r="114">
+      <c r="H114" s="23" t="inlineStr">
+        <is>
+          <t>Q6  基準日セルから5年分（60か月）の月初（1日）を横1行にスピルする</t>
+        </is>
+      </c>
+      <c r="I114" s="13" t="n"/>
+      <c r="J114" s="13" t="n"/>
+      <c r="K114" s="13" t="n"/>
+      <c r="L114" s="14" t="n"/>
+      <c r="M114" s="24" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="21">
-    <mergeCell ref="B126:F126"/>
-    <mergeCell ref="B129:F129"/>
-    <mergeCell ref="B125:F125"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="B22:F22"/>
-    <mergeCell ref="I127:K127"/>
-    <mergeCell ref="I130:K130"/>
-    <mergeCell ref="B96:F96"/>
-    <mergeCell ref="B58:F58"/>
-    <mergeCell ref="B70:F70"/>
-    <mergeCell ref="B130:F130"/>
-    <mergeCell ref="B82:F82"/>
-    <mergeCell ref="B34:F34"/>
-    <mergeCell ref="I128:K128"/>
-    <mergeCell ref="B128:F128"/>
-    <mergeCell ref="B127:F127"/>
-    <mergeCell ref="B124:F124"/>
-    <mergeCell ref="I126:K126"/>
-    <mergeCell ref="B110:F110"/>
-    <mergeCell ref="I129:K129"/>
+  <mergeCells count="18">
+    <mergeCell ref="H108:L108"/>
+    <mergeCell ref="H30:L30"/>
+    <mergeCell ref="H114:L114"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="H109:L109"/>
+    <mergeCell ref="H6:L6"/>
+    <mergeCell ref="H42:L42"/>
+    <mergeCell ref="H54:L54"/>
+    <mergeCell ref="H112:L112"/>
+    <mergeCell ref="H18:L18"/>
+    <mergeCell ref="H66:L66"/>
+    <mergeCell ref="H80:L80"/>
+    <mergeCell ref="H102:L102"/>
+    <mergeCell ref="H94:L94"/>
+    <mergeCell ref="H110:L110"/>
+    <mergeCell ref="H113:L113"/>
+    <mergeCell ref="H107:L107"/>
+    <mergeCell ref="H111:L111"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>